<commit_message>
Switch recipient font to Cinzel Medium; keep Brush Script for reference
- Cinzel Medium (OFL) is the new default recipient font: 24 pt single line, 20/22 pt two lines
- New optional recipient_font column to pick another font per certificate
- Brush Script MT kept in Fonts/; font history recorded in SPEC.md

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EGJZuMn2qF4zfBNmjtSjHp
</commit_message>
<xml_diff>
--- a/Generator/certificates.xlsx
+++ b/Generator/certificates.xlsx
@@ -429,8 +429,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K198"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:L198"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
@@ -443,6 +443,7 @@
     <col width="28" customWidth="1" min="9" max="9"/>
     <col width="40" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -501,6 +502,11 @@
           <t>file_name</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>recipient_font</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -519,10 +525,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>20.6</v>
+        <v>20</v>
       </c>
       <c r="E2" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>46277</v>
@@ -560,10 +566,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>20.6</v>
+        <v>20</v>
       </c>
       <c r="E3" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>46277</v>
@@ -1185,8 +1191,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="120" customWidth="1" min="2" max="2"/>
@@ -1224,7 +1230,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Main recipient line, e.g. company or person. Brush Script MT.</t>
+          <t>Main recipient line, e.g. company or person. Font: Cinzel Medium (all capitals; lowercase letters print as small capitals).</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1254,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Optional font size in pt. Defaults: 30 pt for a single line, 26 pt each for two lines. Too-wide names are shrunk automatically to fit the gold line.</t>
+          <t>Optional font size in pt. Cinzel defaults: 24 pt for a single line; 20 pt over 22 pt for two lines. Too-wide names are shrunk automatically to fit the gold line.</t>
         </is>
       </c>
     </row>
@@ -1325,28 +1331,40 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr"/>
-      <c r="B12" s="3" t="inlineStr"/>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>recipient_font</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Optional. Font file in the Fonts folder for this row only. Leave blank for Cinzel. Previous font, kept for reference: "Brush Script.ttf" (Brush Script MT; sizes used: 30 pt single line, 20.6 pt / 26 pt two lines).</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Limits</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Layout A: 2 Chinese lines, 3 English lines.  Layout B: 3 Chinese lines (incl. the date line), 3 English lines (incl. the date line).</t>
-        </is>
-      </c>
+      <c r="A13" s="3" t="inlineStr"/>
+      <c r="B13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>Limits</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Layout A: 2 Chinese lines, 3 English lines.  Layout B: 3 Chinese lines (incl. the date line), 3 English lines (incl. the date line).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>Output</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>OB-Cert/Output: a JPG (2480x3508 px, 300 dpi) and an A4 PDF per row, plus one combined PDF of all rows for printing.</t>
         </is>

</xml_diff>